<commit_message>
fix: skills tests passed
</commit_message>
<xml_diff>
--- a/evaluation/rag_benchmark/results/rag_benchmark_para_pasar_a_gem.xlsx
+++ b/evaluation/rag_benchmark/results/rag_benchmark_para_pasar_a_gem.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\irene\Desktop\UNIVERSIDAD\TFG\TFG-Tutor-Virtual\evaluation\rag_benchmark\results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4891E41E-BC48-4130-B5EC-B6BC6170C1BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78A66668-E278-45EB-AFCF-AC95E1CB67B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4980" yWindow="3360" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2688" yWindow="2688" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Results_qwen2.5_latest" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2059" uniqueCount="776">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2058" uniqueCount="775">
   <si>
     <t>ID</t>
   </si>
@@ -1447,9 +1447,6 @@
   </si>
   <si>
     <t>RAG</t>
-  </si>
-  <si>
-    <t>Respuestas del gem</t>
   </si>
   <si>
     <t>Estás cerca. Piensa en qué más podría influir. esas resistencias como las que contribuyen a la diferencia de potencial entre N2 y 0.
@@ -2557,7 +2554,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2569,6 +2566,21 @@
       <b/>
       <sz val="11"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <u/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -2606,14 +2618,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2916,13 +2929,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:V553"/>
+  <dimension ref="A1:U553"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="20" max="20" width="59.33203125" customWidth="1"/>
+    <col min="20" max="20" width="8.88671875" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2978,13 +2991,10 @@
         <v>17</v>
       </c>
       <c r="S1" s="1"/>
-      <c r="T1" s="1" t="s">
-        <v>445</v>
-      </c>
+      <c r="T1" s="2"/>
       <c r="U1" s="1"/>
-      <c r="V1" s="1"/>
-    </row>
-    <row r="2" spans="1:22" x14ac:dyDescent="0.3">
+    </row>
+    <row r="2" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1</v>
       </c>
@@ -3040,9 +3050,8 @@
       <c r="R2">
         <v>1</v>
       </c>
-      <c r="T2" s="2"/>
-    </row>
-    <row r="3" spans="1:22" x14ac:dyDescent="0.3">
+    </row>
+    <row r="3" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>2</v>
       </c>
@@ -3099,7 +3108,7 @@
         <v>0.66700000000000004</v>
       </c>
     </row>
-    <row r="4" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>3</v>
       </c>
@@ -3156,7 +3165,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>4</v>
       </c>
@@ -3213,7 +3222,7 @@
         <v>0.66700000000000004</v>
       </c>
     </row>
-    <row r="6" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>5</v>
       </c>
@@ -3270,7 +3279,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>6</v>
       </c>
@@ -3327,7 +3336,7 @@
         <v>0.66700000000000004</v>
       </c>
     </row>
-    <row r="8" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>7</v>
       </c>
@@ -3384,7 +3393,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="9" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>8</v>
       </c>
@@ -3441,7 +3450,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>9</v>
       </c>
@@ -3498,7 +3507,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>10</v>
       </c>
@@ -3555,7 +3564,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>11</v>
       </c>
@@ -3612,7 +3621,7 @@
         <v>0.66700000000000004</v>
       </c>
     </row>
-    <row r="13" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>12</v>
       </c>
@@ -3669,7 +3678,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="14" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>13</v>
       </c>
@@ -3726,7 +3735,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="15" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>14</v>
       </c>
@@ -3783,7 +3792,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>15</v>
       </c>
@@ -14084,7 +14093,7 @@
         <v>90</v>
       </c>
       <c r="E200" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
       <c r="F200">
         <v>4</v>
@@ -14137,7 +14146,7 @@
         <v>90</v>
       </c>
       <c r="E201" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
       <c r="F201">
         <v>4</v>
@@ -14190,7 +14199,7 @@
         <v>90</v>
       </c>
       <c r="E202" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="F202">
         <v>4</v>
@@ -14243,7 +14252,7 @@
         <v>90</v>
       </c>
       <c r="E203" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="F203">
         <v>3</v>
@@ -14296,7 +14305,7 @@
         <v>88</v>
       </c>
       <c r="E204" t="s">
-        <v>450</v>
+        <v>449</v>
       </c>
       <c r="F204">
         <v>4</v>
@@ -14349,10 +14358,10 @@
         <v>1</v>
       </c>
       <c r="D205" t="s">
+        <v>450</v>
+      </c>
+      <c r="E205" t="s">
         <v>451</v>
-      </c>
-      <c r="E205" t="s">
-        <v>452</v>
       </c>
       <c r="F205">
         <v>5</v>
@@ -14461,7 +14470,7 @@
         <v>93</v>
       </c>
       <c r="E207" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="F207">
         <v>4</v>
@@ -14514,10 +14523,10 @@
         <v>1</v>
       </c>
       <c r="D208" t="s">
+        <v>453</v>
+      </c>
+      <c r="E208" t="s">
         <v>454</v>
-      </c>
-      <c r="E208" t="s">
-        <v>455</v>
       </c>
       <c r="F208">
         <v>4</v>
@@ -14567,10 +14576,10 @@
         <v>1</v>
       </c>
       <c r="D209" t="s">
+        <v>455</v>
+      </c>
+      <c r="E209" t="s">
         <v>456</v>
-      </c>
-      <c r="E209" t="s">
-        <v>457</v>
       </c>
       <c r="F209">
         <v>5</v>
@@ -14623,10 +14632,10 @@
         <v>1</v>
       </c>
       <c r="D210" t="s">
+        <v>457</v>
+      </c>
+      <c r="E210" t="s">
         <v>458</v>
-      </c>
-      <c r="E210" t="s">
-        <v>459</v>
       </c>
       <c r="F210">
         <v>4</v>
@@ -14676,10 +14685,10 @@
         <v>1</v>
       </c>
       <c r="D211" t="s">
+        <v>459</v>
+      </c>
+      <c r="E211" t="s">
         <v>460</v>
-      </c>
-      <c r="E211" t="s">
-        <v>461</v>
       </c>
       <c r="F211">
         <v>3</v>
@@ -14732,7 +14741,7 @@
         <v>90</v>
       </c>
       <c r="E212" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="F212">
         <v>4</v>
@@ -14785,7 +14794,7 @@
         <v>90</v>
       </c>
       <c r="E213" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="F213">
         <v>3</v>
@@ -14838,7 +14847,7 @@
         <v>90</v>
       </c>
       <c r="E214" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
       <c r="F214">
         <v>3</v>
@@ -14891,7 +14900,7 @@
         <v>90</v>
       </c>
       <c r="E215" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
       <c r="F215">
         <v>3</v>
@@ -14944,7 +14953,7 @@
         <v>90</v>
       </c>
       <c r="E216" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="F216">
         <v>3</v>
@@ -14997,7 +15006,7 @@
         <v>90</v>
       </c>
       <c r="E217" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="F217">
         <v>3</v>
@@ -15050,7 +15059,7 @@
         <v>88</v>
       </c>
       <c r="E218" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="F218">
         <v>3</v>
@@ -15103,10 +15112,10 @@
         <v>1</v>
       </c>
       <c r="D219" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
       <c r="E219" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="F219">
         <v>3</v>
@@ -15162,7 +15171,7 @@
         <v>95</v>
       </c>
       <c r="E220" t="s">
-        <v>470</v>
+        <v>469</v>
       </c>
       <c r="F220">
         <v>3</v>
@@ -15218,7 +15227,7 @@
         <v>93</v>
       </c>
       <c r="E221" t="s">
-        <v>471</v>
+        <v>470</v>
       </c>
       <c r="F221">
         <v>3</v>
@@ -15271,10 +15280,10 @@
         <v>1</v>
       </c>
       <c r="D222" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
       <c r="E222" t="s">
-        <v>472</v>
+        <v>471</v>
       </c>
       <c r="F222">
         <v>3</v>
@@ -15327,10 +15336,10 @@
         <v>1</v>
       </c>
       <c r="D223" t="s">
-        <v>456</v>
+        <v>455</v>
       </c>
       <c r="E223" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
       <c r="F223">
         <v>4</v>
@@ -15383,10 +15392,10 @@
         <v>1</v>
       </c>
       <c r="D224" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="E224" t="s">
-        <v>474</v>
+        <v>473</v>
       </c>
       <c r="F224">
         <v>3</v>
@@ -15439,10 +15448,10 @@
         <v>1</v>
       </c>
       <c r="D225" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="E225" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
       <c r="F225">
         <v>3</v>
@@ -15498,7 +15507,7 @@
         <v>90</v>
       </c>
       <c r="E226" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
       <c r="F226">
         <v>3</v>
@@ -15551,7 +15560,7 @@
         <v>90</v>
       </c>
       <c r="E227" t="s">
-        <v>477</v>
+        <v>476</v>
       </c>
       <c r="F227">
         <v>3</v>
@@ -15604,7 +15613,7 @@
         <v>105</v>
       </c>
       <c r="E228" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="F228">
         <v>3</v>
@@ -15660,7 +15669,7 @@
         <v>108</v>
       </c>
       <c r="E229" t="s">
-        <v>479</v>
+        <v>478</v>
       </c>
       <c r="F229">
         <v>3</v>
@@ -15716,7 +15725,7 @@
         <v>110</v>
       </c>
       <c r="E230" t="s">
-        <v>480</v>
+        <v>479</v>
       </c>
       <c r="F230">
         <v>3</v>
@@ -15772,7 +15781,7 @@
         <v>112</v>
       </c>
       <c r="E231" t="s">
-        <v>481</v>
+        <v>480</v>
       </c>
       <c r="F231">
         <v>4</v>
@@ -15825,10 +15834,10 @@
         <v>3</v>
       </c>
       <c r="D232" t="s">
+        <v>481</v>
+      </c>
+      <c r="E232" t="s">
         <v>482</v>
-      </c>
-      <c r="E232" t="s">
-        <v>483</v>
       </c>
       <c r="F232">
         <v>5</v>
@@ -15875,10 +15884,10 @@
         <v>3</v>
       </c>
       <c r="D233" t="s">
+        <v>483</v>
+      </c>
+      <c r="E233" t="s">
         <v>484</v>
-      </c>
-      <c r="E233" t="s">
-        <v>485</v>
       </c>
       <c r="F233">
         <v>4</v>
@@ -15928,10 +15937,10 @@
         <v>3</v>
       </c>
       <c r="D234" t="s">
+        <v>485</v>
+      </c>
+      <c r="E234" t="s">
         <v>486</v>
-      </c>
-      <c r="E234" t="s">
-        <v>487</v>
       </c>
       <c r="F234">
         <v>5</v>
@@ -15984,7 +15993,7 @@
         <v>121</v>
       </c>
       <c r="E235" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="F235">
         <v>5</v>
@@ -16040,7 +16049,7 @@
         <v>124</v>
       </c>
       <c r="E236" t="s">
-        <v>489</v>
+        <v>488</v>
       </c>
       <c r="F236">
         <v>5</v>
@@ -16096,7 +16105,7 @@
         <v>126</v>
       </c>
       <c r="E237" t="s">
-        <v>490</v>
+        <v>489</v>
       </c>
       <c r="F237">
         <v>3</v>
@@ -16152,7 +16161,7 @@
         <v>128</v>
       </c>
       <c r="E238" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
       <c r="F238">
         <v>4</v>
@@ -16208,7 +16217,7 @@
         <v>131</v>
       </c>
       <c r="E239" t="s">
-        <v>492</v>
+        <v>491</v>
       </c>
       <c r="F239">
         <v>4</v>
@@ -16264,7 +16273,7 @@
         <v>133</v>
       </c>
       <c r="E240" t="s">
-        <v>493</v>
+        <v>492</v>
       </c>
       <c r="F240">
         <v>4</v>
@@ -16320,7 +16329,7 @@
         <v>135</v>
       </c>
       <c r="E241" t="s">
-        <v>494</v>
+        <v>493</v>
       </c>
       <c r="F241">
         <v>4</v>
@@ -16376,7 +16385,7 @@
         <v>137</v>
       </c>
       <c r="E242" t="s">
-        <v>495</v>
+        <v>494</v>
       </c>
       <c r="F242">
         <v>4</v>
@@ -16432,7 +16441,7 @@
         <v>139</v>
       </c>
       <c r="E243" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
       <c r="F243">
         <v>4</v>
@@ -16485,10 +16494,10 @@
         <v>3</v>
       </c>
       <c r="D244" t="s">
+        <v>496</v>
+      </c>
+      <c r="E244" t="s">
         <v>497</v>
-      </c>
-      <c r="E244" t="s">
-        <v>498</v>
       </c>
       <c r="F244">
         <v>3</v>
@@ -16541,10 +16550,10 @@
         <v>3</v>
       </c>
       <c r="D245" t="s">
+        <v>498</v>
+      </c>
+      <c r="E245" t="s">
         <v>499</v>
-      </c>
-      <c r="E245" t="s">
-        <v>500</v>
       </c>
       <c r="F245">
         <v>4</v>
@@ -16597,10 +16606,10 @@
         <v>3</v>
       </c>
       <c r="D246" t="s">
+        <v>500</v>
+      </c>
+      <c r="E246" t="s">
         <v>501</v>
-      </c>
-      <c r="E246" t="s">
-        <v>502</v>
       </c>
       <c r="F246">
         <v>4</v>
@@ -16656,7 +16665,7 @@
         <v>147</v>
       </c>
       <c r="E247" t="s">
-        <v>503</v>
+        <v>502</v>
       </c>
       <c r="F247">
         <v>4</v>
@@ -16712,7 +16721,7 @@
         <v>149</v>
       </c>
       <c r="E248" t="s">
-        <v>504</v>
+        <v>503</v>
       </c>
       <c r="F248">
         <v>5</v>
@@ -16768,7 +16777,7 @@
         <v>151</v>
       </c>
       <c r="E249" t="s">
-        <v>505</v>
+        <v>504</v>
       </c>
       <c r="F249">
         <v>4</v>
@@ -16824,7 +16833,7 @@
         <v>153</v>
       </c>
       <c r="E250" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
       <c r="F250">
         <v>3</v>
@@ -16880,7 +16889,7 @@
         <v>155</v>
       </c>
       <c r="E251" t="s">
-        <v>507</v>
+        <v>506</v>
       </c>
       <c r="F251">
         <v>4</v>
@@ -16936,7 +16945,7 @@
         <v>157</v>
       </c>
       <c r="E252" t="s">
-        <v>508</v>
+        <v>507</v>
       </c>
       <c r="F252">
         <v>5</v>
@@ -16992,7 +17001,7 @@
         <v>159</v>
       </c>
       <c r="E253" t="s">
-        <v>509</v>
+        <v>508</v>
       </c>
       <c r="F253">
         <v>4</v>
@@ -17048,7 +17057,7 @@
         <v>161</v>
       </c>
       <c r="E254" t="s">
-        <v>510</v>
+        <v>509</v>
       </c>
       <c r="F254">
         <v>3</v>
@@ -17104,7 +17113,7 @@
         <v>163</v>
       </c>
       <c r="E255" t="s">
-        <v>511</v>
+        <v>510</v>
       </c>
       <c r="F255">
         <v>3</v>
@@ -17160,7 +17169,7 @@
         <v>165</v>
       </c>
       <c r="E256" t="s">
-        <v>512</v>
+        <v>511</v>
       </c>
       <c r="F256">
         <v>2</v>
@@ -17216,7 +17225,7 @@
         <v>167</v>
       </c>
       <c r="E257" t="s">
-        <v>513</v>
+        <v>512</v>
       </c>
       <c r="F257">
         <v>4</v>
@@ -17272,7 +17281,7 @@
         <v>168</v>
       </c>
       <c r="E258" t="s">
-        <v>514</v>
+        <v>513</v>
       </c>
       <c r="F258">
         <v>4</v>
@@ -17328,7 +17337,7 @@
         <v>170</v>
       </c>
       <c r="E259" t="s">
-        <v>515</v>
+        <v>514</v>
       </c>
       <c r="F259">
         <v>3</v>
@@ -17384,7 +17393,7 @@
         <v>172</v>
       </c>
       <c r="E260" t="s">
-        <v>516</v>
+        <v>515</v>
       </c>
       <c r="F260">
         <v>4</v>
@@ -17440,7 +17449,7 @@
         <v>174</v>
       </c>
       <c r="E261" t="s">
-        <v>517</v>
+        <v>516</v>
       </c>
       <c r="F261">
         <v>5</v>
@@ -17493,7 +17502,7 @@
         <v>176</v>
       </c>
       <c r="E262" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
       <c r="F262">
         <v>4</v>
@@ -17549,7 +17558,7 @@
         <v>177</v>
       </c>
       <c r="E263" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
       <c r="F263">
         <v>5</v>
@@ -17602,7 +17611,7 @@
         <v>179</v>
       </c>
       <c r="E264" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
       <c r="F264">
         <v>3</v>
@@ -17655,7 +17664,7 @@
         <v>181</v>
       </c>
       <c r="E265" t="s">
-        <v>521</v>
+        <v>520</v>
       </c>
       <c r="F265">
         <v>4</v>
@@ -17708,7 +17717,7 @@
         <v>105</v>
       </c>
       <c r="E266" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
       <c r="F266">
         <v>2</v>
@@ -17764,7 +17773,7 @@
         <v>108</v>
       </c>
       <c r="E267" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
       <c r="F267">
         <v>4</v>
@@ -17820,7 +17829,7 @@
         <v>110</v>
       </c>
       <c r="E268" t="s">
-        <v>524</v>
+        <v>523</v>
       </c>
       <c r="F268">
         <v>3</v>
@@ -17876,7 +17885,7 @@
         <v>112</v>
       </c>
       <c r="E269" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="F269">
         <v>5</v>
@@ -17926,10 +17935,10 @@
         <v>3</v>
       </c>
       <c r="D270" t="s">
-        <v>482</v>
+        <v>481</v>
       </c>
       <c r="E270" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="F270">
         <v>5</v>
@@ -17979,10 +17988,10 @@
         <v>3</v>
       </c>
       <c r="D271" t="s">
-        <v>484</v>
+        <v>483</v>
       </c>
       <c r="E271" t="s">
-        <v>527</v>
+        <v>526</v>
       </c>
       <c r="F271">
         <v>3</v>
@@ -18032,10 +18041,10 @@
         <v>3</v>
       </c>
       <c r="D272" t="s">
-        <v>486</v>
+        <v>485</v>
       </c>
       <c r="E272" t="s">
-        <v>528</v>
+        <v>527</v>
       </c>
       <c r="F272">
         <v>3</v>
@@ -18088,7 +18097,7 @@
         <v>121</v>
       </c>
       <c r="E273" t="s">
-        <v>529</v>
+        <v>528</v>
       </c>
       <c r="F273">
         <v>4</v>
@@ -18144,7 +18153,7 @@
         <v>124</v>
       </c>
       <c r="E274" t="s">
-        <v>530</v>
+        <v>529</v>
       </c>
       <c r="F274">
         <v>4</v>
@@ -18200,7 +18209,7 @@
         <v>126</v>
       </c>
       <c r="E275" t="s">
-        <v>531</v>
+        <v>530</v>
       </c>
       <c r="F275">
         <v>4</v>
@@ -18256,7 +18265,7 @@
         <v>128</v>
       </c>
       <c r="E276" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="F276">
         <v>4</v>
@@ -18312,7 +18321,7 @@
         <v>131</v>
       </c>
       <c r="E277" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="F277">
         <v>4</v>
@@ -18368,7 +18377,7 @@
         <v>133</v>
       </c>
       <c r="E278" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="F278">
         <v>4</v>
@@ -18424,7 +18433,7 @@
         <v>135</v>
       </c>
       <c r="E279" t="s">
-        <v>535</v>
+        <v>534</v>
       </c>
       <c r="F279">
         <v>3</v>
@@ -18480,7 +18489,7 @@
         <v>137</v>
       </c>
       <c r="E280" t="s">
-        <v>536</v>
+        <v>535</v>
       </c>
       <c r="F280">
         <v>4</v>
@@ -18536,7 +18545,7 @@
         <v>139</v>
       </c>
       <c r="E281" t="s">
-        <v>537</v>
+        <v>536</v>
       </c>
       <c r="F281">
         <v>5</v>
@@ -18589,10 +18598,10 @@
         <v>3</v>
       </c>
       <c r="D282" t="s">
-        <v>497</v>
+        <v>496</v>
       </c>
       <c r="E282" t="s">
-        <v>538</v>
+        <v>537</v>
       </c>
       <c r="F282">
         <v>5</v>
@@ -18645,10 +18654,10 @@
         <v>3</v>
       </c>
       <c r="D283" t="s">
-        <v>499</v>
+        <v>498</v>
       </c>
       <c r="E283" t="s">
-        <v>539</v>
+        <v>538</v>
       </c>
       <c r="F283">
         <v>2</v>
@@ -18701,10 +18710,10 @@
         <v>3</v>
       </c>
       <c r="D284" t="s">
-        <v>501</v>
+        <v>500</v>
       </c>
       <c r="E284" t="s">
-        <v>540</v>
+        <v>539</v>
       </c>
       <c r="F284">
         <v>4</v>
@@ -18760,7 +18769,7 @@
         <v>147</v>
       </c>
       <c r="E285" t="s">
-        <v>541</v>
+        <v>540</v>
       </c>
       <c r="F285">
         <v>5</v>
@@ -18816,7 +18825,7 @@
         <v>149</v>
       </c>
       <c r="E286" t="s">
-        <v>542</v>
+        <v>541</v>
       </c>
       <c r="F286">
         <v>3</v>
@@ -18872,7 +18881,7 @@
         <v>151</v>
       </c>
       <c r="E287" t="s">
-        <v>543</v>
+        <v>542</v>
       </c>
       <c r="F287">
         <v>5</v>
@@ -18928,7 +18937,7 @@
         <v>153</v>
       </c>
       <c r="E288" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
       <c r="F288">
         <v>5</v>
@@ -18984,7 +18993,7 @@
         <v>155</v>
       </c>
       <c r="E289" t="s">
-        <v>545</v>
+        <v>544</v>
       </c>
       <c r="F289">
         <v>4</v>
@@ -19040,7 +19049,7 @@
         <v>157</v>
       </c>
       <c r="E290" t="s">
-        <v>546</v>
+        <v>545</v>
       </c>
       <c r="F290">
         <v>3</v>
@@ -19096,7 +19105,7 @@
         <v>159</v>
       </c>
       <c r="E291" t="s">
-        <v>547</v>
+        <v>546</v>
       </c>
       <c r="F291">
         <v>4</v>
@@ -19152,7 +19161,7 @@
         <v>161</v>
       </c>
       <c r="E292" t="s">
-        <v>548</v>
+        <v>547</v>
       </c>
       <c r="F292">
         <v>5</v>
@@ -19205,7 +19214,7 @@
         <v>163</v>
       </c>
       <c r="E293" t="s">
-        <v>549</v>
+        <v>548</v>
       </c>
       <c r="F293">
         <v>5</v>
@@ -19261,7 +19270,7 @@
         <v>165</v>
       </c>
       <c r="E294" t="s">
-        <v>550</v>
+        <v>549</v>
       </c>
       <c r="F294">
         <v>4</v>
@@ -19317,7 +19326,7 @@
         <v>167</v>
       </c>
       <c r="E295" t="s">
-        <v>551</v>
+        <v>550</v>
       </c>
       <c r="F295">
         <v>4</v>
@@ -19373,7 +19382,7 @@
         <v>168</v>
       </c>
       <c r="E296" t="s">
-        <v>552</v>
+        <v>551</v>
       </c>
       <c r="F296">
         <v>3</v>
@@ -19429,7 +19438,7 @@
         <v>170</v>
       </c>
       <c r="E297" t="s">
-        <v>553</v>
+        <v>552</v>
       </c>
       <c r="F297">
         <v>4</v>
@@ -19485,7 +19494,7 @@
         <v>172</v>
       </c>
       <c r="E298" t="s">
-        <v>554</v>
+        <v>553</v>
       </c>
       <c r="F298">
         <v>4</v>
@@ -19541,7 +19550,7 @@
         <v>174</v>
       </c>
       <c r="E299" t="s">
-        <v>555</v>
+        <v>554</v>
       </c>
       <c r="F299">
         <v>5</v>
@@ -19597,7 +19606,7 @@
         <v>176</v>
       </c>
       <c r="E300" t="s">
-        <v>556</v>
+        <v>555</v>
       </c>
       <c r="F300">
         <v>4</v>
@@ -19653,7 +19662,7 @@
         <v>177</v>
       </c>
       <c r="E301" t="s">
-        <v>557</v>
+        <v>556</v>
       </c>
       <c r="F301">
         <v>5</v>
@@ -19709,7 +19718,7 @@
         <v>179</v>
       </c>
       <c r="E302" t="s">
-        <v>558</v>
+        <v>557</v>
       </c>
       <c r="F302">
         <v>5</v>
@@ -19762,7 +19771,7 @@
         <v>181</v>
       </c>
       <c r="E303" t="s">
-        <v>559</v>
+        <v>558</v>
       </c>
       <c r="F303">
         <v>5</v>
@@ -19815,7 +19824,7 @@
         <v>183</v>
       </c>
       <c r="E304" t="s">
-        <v>560</v>
+        <v>559</v>
       </c>
       <c r="F304">
         <v>3</v>
@@ -19871,7 +19880,7 @@
         <v>185</v>
       </c>
       <c r="E305" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="F305">
         <v>4</v>
@@ -19927,7 +19936,7 @@
         <v>187</v>
       </c>
       <c r="E306" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
       <c r="F306">
         <v>4</v>
@@ -19983,7 +19992,7 @@
         <v>189</v>
       </c>
       <c r="E307" t="s">
-        <v>563</v>
+        <v>562</v>
       </c>
       <c r="F307">
         <v>4</v>
@@ -20039,7 +20048,7 @@
         <v>192</v>
       </c>
       <c r="E308" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
       <c r="F308">
         <v>5</v>
@@ -20089,10 +20098,10 @@
         <v>4</v>
       </c>
       <c r="D309" t="s">
+        <v>564</v>
+      </c>
+      <c r="E309" t="s">
         <v>565</v>
-      </c>
-      <c r="E309" t="s">
-        <v>566</v>
       </c>
       <c r="F309">
         <v>5</v>
@@ -20145,7 +20154,7 @@
         <v>196</v>
       </c>
       <c r="E310" t="s">
-        <v>567</v>
+        <v>566</v>
       </c>
       <c r="F310">
         <v>4</v>
@@ -20201,7 +20210,7 @@
         <v>88</v>
       </c>
       <c r="E311" t="s">
-        <v>568</v>
+        <v>567</v>
       </c>
       <c r="F311">
         <v>3</v>
@@ -20254,7 +20263,7 @@
         <v>199</v>
       </c>
       <c r="E312" t="s">
-        <v>569</v>
+        <v>568</v>
       </c>
       <c r="F312">
         <v>4</v>
@@ -20310,7 +20319,7 @@
         <v>200</v>
       </c>
       <c r="E313" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="F313">
         <v>4</v>
@@ -20363,10 +20372,10 @@
         <v>4</v>
       </c>
       <c r="D314" t="s">
+        <v>570</v>
+      </c>
+      <c r="E314" t="s">
         <v>571</v>
-      </c>
-      <c r="E314" t="s">
-        <v>572</v>
       </c>
       <c r="F314">
         <v>4</v>
@@ -20422,7 +20431,7 @@
         <v>205</v>
       </c>
       <c r="E315" t="s">
-        <v>573</v>
+        <v>572</v>
       </c>
       <c r="F315">
         <v>5</v>
@@ -20478,7 +20487,7 @@
         <v>207</v>
       </c>
       <c r="E316" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
       <c r="F316">
         <v>4</v>
@@ -20534,7 +20543,7 @@
         <v>209</v>
       </c>
       <c r="E317" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
       <c r="F317">
         <v>3</v>
@@ -20587,7 +20596,7 @@
         <v>211</v>
       </c>
       <c r="E318" t="s">
-        <v>576</v>
+        <v>575</v>
       </c>
       <c r="F318">
         <v>5</v>
@@ -20643,7 +20652,7 @@
         <v>213</v>
       </c>
       <c r="E319" t="s">
-        <v>577</v>
+        <v>576</v>
       </c>
       <c r="F319">
         <v>5</v>
@@ -20699,7 +20708,7 @@
         <v>215</v>
       </c>
       <c r="E320" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="F320">
         <v>3</v>
@@ -20755,7 +20764,7 @@
         <v>218</v>
       </c>
       <c r="E321" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
       <c r="F321">
         <v>1</v>
@@ -20811,7 +20820,7 @@
         <v>220</v>
       </c>
       <c r="E322" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="F322">
         <v>2</v>
@@ -20867,7 +20876,7 @@
         <v>222</v>
       </c>
       <c r="E323" t="s">
-        <v>581</v>
+        <v>580</v>
       </c>
       <c r="F323">
         <v>2</v>
@@ -20920,7 +20929,7 @@
         <v>224</v>
       </c>
       <c r="E324" t="s">
-        <v>582</v>
+        <v>581</v>
       </c>
       <c r="F324">
         <v>4</v>
@@ -20973,10 +20982,10 @@
         <v>4</v>
       </c>
       <c r="D325" t="s">
+        <v>582</v>
+      </c>
+      <c r="E325" t="s">
         <v>583</v>
-      </c>
-      <c r="E325" t="s">
-        <v>584</v>
       </c>
       <c r="F325">
         <v>4</v>
@@ -21029,10 +21038,10 @@
         <v>4</v>
       </c>
       <c r="D326" t="s">
+        <v>584</v>
+      </c>
+      <c r="E326" t="s">
         <v>585</v>
-      </c>
-      <c r="E326" t="s">
-        <v>586</v>
       </c>
       <c r="F326">
         <v>1</v>
@@ -21088,7 +21097,7 @@
         <v>231</v>
       </c>
       <c r="E327" t="s">
-        <v>587</v>
+        <v>586</v>
       </c>
       <c r="F327">
         <v>4</v>
@@ -21144,7 +21153,7 @@
         <v>233</v>
       </c>
       <c r="E328" t="s">
-        <v>588</v>
+        <v>587</v>
       </c>
       <c r="F328">
         <v>3</v>
@@ -21197,7 +21206,7 @@
         <v>235</v>
       </c>
       <c r="E329" t="s">
-        <v>589</v>
+        <v>588</v>
       </c>
       <c r="F329">
         <v>4</v>
@@ -21253,7 +21262,7 @@
         <v>238</v>
       </c>
       <c r="E330" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="F330">
         <v>3</v>
@@ -21309,7 +21318,7 @@
         <v>240</v>
       </c>
       <c r="E331" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="F331">
         <v>4</v>
@@ -21362,10 +21371,10 @@
         <v>4</v>
       </c>
       <c r="D332" t="s">
+        <v>591</v>
+      </c>
+      <c r="E332" t="s">
         <v>592</v>
-      </c>
-      <c r="E332" t="s">
-        <v>593</v>
       </c>
       <c r="F332">
         <v>4</v>
@@ -21421,7 +21430,7 @@
         <v>244</v>
       </c>
       <c r="E333" t="s">
-        <v>594</v>
+        <v>593</v>
       </c>
       <c r="F333">
         <v>2</v>
@@ -21477,7 +21486,7 @@
         <v>246</v>
       </c>
       <c r="E334" t="s">
-        <v>595</v>
+        <v>594</v>
       </c>
       <c r="F334">
         <v>2</v>
@@ -21533,7 +21542,7 @@
         <v>248</v>
       </c>
       <c r="E335" t="s">
-        <v>596</v>
+        <v>595</v>
       </c>
       <c r="F335">
         <v>4</v>
@@ -21589,7 +21598,7 @@
         <v>250</v>
       </c>
       <c r="E336" t="s">
-        <v>597</v>
+        <v>596</v>
       </c>
       <c r="F336">
         <v>5</v>
@@ -21642,7 +21651,7 @@
         <v>183</v>
       </c>
       <c r="E337" t="s">
-        <v>598</v>
+        <v>597</v>
       </c>
       <c r="F337">
         <v>4</v>
@@ -21698,7 +21707,7 @@
         <v>185</v>
       </c>
       <c r="E338" t="s">
-        <v>599</v>
+        <v>598</v>
       </c>
       <c r="F338">
         <v>4</v>
@@ -21754,7 +21763,7 @@
         <v>187</v>
       </c>
       <c r="E339" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="F339">
         <v>3</v>
@@ -21810,7 +21819,7 @@
         <v>189</v>
       </c>
       <c r="E340" t="s">
-        <v>601</v>
+        <v>600</v>
       </c>
       <c r="F340">
         <v>5</v>
@@ -21863,7 +21872,7 @@
         <v>192</v>
       </c>
       <c r="E341" t="s">
-        <v>602</v>
+        <v>601</v>
       </c>
       <c r="F341">
         <v>4</v>
@@ -21913,10 +21922,10 @@
         <v>4</v>
       </c>
       <c r="D342" t="s">
-        <v>565</v>
+        <v>564</v>
       </c>
       <c r="E342" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="F342">
         <v>3</v>
@@ -21969,7 +21978,7 @@
         <v>196</v>
       </c>
       <c r="E343" t="s">
-        <v>604</v>
+        <v>603</v>
       </c>
       <c r="F343">
         <v>3</v>
@@ -22025,7 +22034,7 @@
         <v>88</v>
       </c>
       <c r="E344" t="s">
-        <v>605</v>
+        <v>604</v>
       </c>
       <c r="F344">
         <v>4</v>
@@ -22078,7 +22087,7 @@
         <v>199</v>
       </c>
       <c r="E345" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="F345">
         <v>4</v>
@@ -22134,7 +22143,7 @@
         <v>200</v>
       </c>
       <c r="E346" t="s">
-        <v>607</v>
+        <v>606</v>
       </c>
       <c r="F346">
         <v>2</v>
@@ -22187,10 +22196,10 @@
         <v>4</v>
       </c>
       <c r="D347" t="s">
-        <v>571</v>
+        <v>570</v>
       </c>
       <c r="E347" t="s">
-        <v>608</v>
+        <v>607</v>
       </c>
       <c r="F347">
         <v>5</v>
@@ -22246,7 +22255,7 @@
         <v>205</v>
       </c>
       <c r="E348" t="s">
-        <v>609</v>
+        <v>608</v>
       </c>
       <c r="F348">
         <v>4</v>
@@ -22302,7 +22311,7 @@
         <v>207</v>
       </c>
       <c r="E349" t="s">
-        <v>610</v>
+        <v>609</v>
       </c>
       <c r="F349">
         <v>4</v>
@@ -22358,7 +22367,7 @@
         <v>209</v>
       </c>
       <c r="E350" t="s">
-        <v>611</v>
+        <v>610</v>
       </c>
       <c r="F350">
         <v>5</v>
@@ -22411,7 +22420,7 @@
         <v>211</v>
       </c>
       <c r="E351" t="s">
-        <v>612</v>
+        <v>611</v>
       </c>
       <c r="F351">
         <v>3</v>
@@ -22467,7 +22476,7 @@
         <v>213</v>
       </c>
       <c r="E352" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="F352">
         <v>3</v>
@@ -22523,7 +22532,7 @@
         <v>215</v>
       </c>
       <c r="E353" t="s">
-        <v>614</v>
+        <v>613</v>
       </c>
       <c r="F353">
         <v>4</v>
@@ -22576,7 +22585,7 @@
         <v>218</v>
       </c>
       <c r="E354" t="s">
-        <v>615</v>
+        <v>614</v>
       </c>
       <c r="F354">
         <v>4</v>
@@ -22632,7 +22641,7 @@
         <v>220</v>
       </c>
       <c r="E355" t="s">
-        <v>616</v>
+        <v>615</v>
       </c>
       <c r="F355">
         <v>4</v>
@@ -22688,7 +22697,7 @@
         <v>222</v>
       </c>
       <c r="E356" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
       <c r="F356">
         <v>4</v>
@@ -22741,7 +22750,7 @@
         <v>224</v>
       </c>
       <c r="E357" t="s">
-        <v>618</v>
+        <v>617</v>
       </c>
       <c r="F357">
         <v>4</v>
@@ -22794,10 +22803,10 @@
         <v>4</v>
       </c>
       <c r="D358" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
       <c r="E358" t="s">
-        <v>619</v>
+        <v>618</v>
       </c>
       <c r="F358">
         <v>5</v>
@@ -22850,10 +22859,10 @@
         <v>4</v>
       </c>
       <c r="D359" t="s">
-        <v>585</v>
+        <v>584</v>
       </c>
       <c r="E359" t="s">
-        <v>620</v>
+        <v>619</v>
       </c>
       <c r="F359">
         <v>4</v>
@@ -22909,7 +22918,7 @@
         <v>231</v>
       </c>
       <c r="E360" t="s">
-        <v>621</v>
+        <v>620</v>
       </c>
       <c r="F360">
         <v>5</v>
@@ -22965,7 +22974,7 @@
         <v>233</v>
       </c>
       <c r="E361" t="s">
-        <v>622</v>
+        <v>621</v>
       </c>
       <c r="F361">
         <v>5</v>
@@ -23021,7 +23030,7 @@
         <v>235</v>
       </c>
       <c r="E362" t="s">
-        <v>623</v>
+        <v>622</v>
       </c>
       <c r="F362">
         <v>3</v>
@@ -23077,7 +23086,7 @@
         <v>238</v>
       </c>
       <c r="E363" t="s">
-        <v>624</v>
+        <v>623</v>
       </c>
       <c r="F363">
         <v>4</v>
@@ -23133,7 +23142,7 @@
         <v>240</v>
       </c>
       <c r="E364" t="s">
-        <v>625</v>
+        <v>624</v>
       </c>
       <c r="F364">
         <v>3</v>
@@ -23186,10 +23195,10 @@
         <v>4</v>
       </c>
       <c r="D365" t="s">
-        <v>592</v>
+        <v>591</v>
       </c>
       <c r="E365" t="s">
-        <v>626</v>
+        <v>625</v>
       </c>
       <c r="F365">
         <v>4</v>
@@ -23245,7 +23254,7 @@
         <v>244</v>
       </c>
       <c r="E366" t="s">
-        <v>627</v>
+        <v>626</v>
       </c>
       <c r="F366">
         <v>4</v>
@@ -23301,7 +23310,7 @@
         <v>246</v>
       </c>
       <c r="E367" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
       <c r="F367">
         <v>3</v>
@@ -23357,7 +23366,7 @@
         <v>248</v>
       </c>
       <c r="E368" t="s">
-        <v>629</v>
+        <v>628</v>
       </c>
       <c r="F368">
         <v>5</v>
@@ -23413,7 +23422,7 @@
         <v>250</v>
       </c>
       <c r="E369" t="s">
-        <v>630</v>
+        <v>629</v>
       </c>
       <c r="F369">
         <v>5</v>
@@ -23466,7 +23475,7 @@
         <v>209</v>
       </c>
       <c r="E370" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="F370">
         <v>3</v>
@@ -23522,7 +23531,7 @@
         <v>194</v>
       </c>
       <c r="E371" t="s">
-        <v>632</v>
+        <v>631</v>
       </c>
       <c r="F371">
         <v>4</v>
@@ -23578,7 +23587,7 @@
         <v>254</v>
       </c>
       <c r="E372" t="s">
-        <v>633</v>
+        <v>632</v>
       </c>
       <c r="F372">
         <v>3</v>
@@ -23737,7 +23746,7 @@
         <v>259</v>
       </c>
       <c r="E375" t="s">
-        <v>634</v>
+        <v>633</v>
       </c>
       <c r="F375">
         <v>4</v>
@@ -23790,7 +23799,7 @@
         <v>261</v>
       </c>
       <c r="E376" t="s">
-        <v>635</v>
+        <v>634</v>
       </c>
       <c r="F376">
         <v>4</v>
@@ -23843,7 +23852,7 @@
         <v>263</v>
       </c>
       <c r="E377" t="s">
-        <v>636</v>
+        <v>635</v>
       </c>
       <c r="F377">
         <v>3</v>
@@ -23896,7 +23905,7 @@
         <v>265</v>
       </c>
       <c r="E378" t="s">
-        <v>637</v>
+        <v>636</v>
       </c>
       <c r="F378">
         <v>1</v>
@@ -23949,7 +23958,7 @@
         <v>267</v>
       </c>
       <c r="E379" t="s">
-        <v>638</v>
+        <v>637</v>
       </c>
       <c r="F379">
         <v>1</v>
@@ -24005,7 +24014,7 @@
         <v>269</v>
       </c>
       <c r="E380" t="s">
-        <v>639</v>
+        <v>638</v>
       </c>
       <c r="F380">
         <v>5</v>
@@ -24061,7 +24070,7 @@
         <v>271</v>
       </c>
       <c r="E381" t="s">
-        <v>640</v>
+        <v>639</v>
       </c>
       <c r="F381">
         <v>3</v>
@@ -24114,7 +24123,7 @@
         <v>177</v>
       </c>
       <c r="E382" t="s">
-        <v>641</v>
+        <v>640</v>
       </c>
       <c r="F382">
         <v>4</v>
@@ -24167,7 +24176,7 @@
         <v>274</v>
       </c>
       <c r="E383" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="F383">
         <v>5</v>
@@ -24217,7 +24226,7 @@
         <v>276</v>
       </c>
       <c r="E384" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="F384">
         <v>4</v>
@@ -24270,7 +24279,7 @@
         <v>213</v>
       </c>
       <c r="E385" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="F385">
         <v>3</v>
@@ -24326,7 +24335,7 @@
         <v>211</v>
       </c>
       <c r="E386" t="s">
-        <v>645</v>
+        <v>644</v>
       </c>
       <c r="F386">
         <v>2</v>
@@ -24379,7 +24388,7 @@
         <v>280</v>
       </c>
       <c r="E387" t="s">
-        <v>646</v>
+        <v>645</v>
       </c>
       <c r="F387">
         <v>2</v>
@@ -24432,7 +24441,7 @@
         <v>282</v>
       </c>
       <c r="E388" t="s">
-        <v>647</v>
+        <v>646</v>
       </c>
       <c r="F388">
         <v>3</v>
@@ -24485,7 +24494,7 @@
         <v>284</v>
       </c>
       <c r="E389" t="s">
-        <v>648</v>
+        <v>647</v>
       </c>
       <c r="F389">
         <v>3</v>
@@ -24538,7 +24547,7 @@
         <v>286</v>
       </c>
       <c r="E390" t="s">
-        <v>649</v>
+        <v>648</v>
       </c>
       <c r="F390">
         <v>3</v>
@@ -24594,7 +24603,7 @@
         <v>288</v>
       </c>
       <c r="E391" t="s">
-        <v>650</v>
+        <v>649</v>
       </c>
       <c r="F391">
         <v>4</v>
@@ -24647,7 +24656,7 @@
         <v>290</v>
       </c>
       <c r="E392" t="s">
-        <v>651</v>
+        <v>650</v>
       </c>
       <c r="F392">
         <v>5</v>
@@ -24700,7 +24709,7 @@
         <v>292</v>
       </c>
       <c r="E393" t="s">
-        <v>652</v>
+        <v>651</v>
       </c>
       <c r="F393">
         <v>3</v>
@@ -24756,7 +24765,7 @@
         <v>294</v>
       </c>
       <c r="E394" t="s">
-        <v>653</v>
+        <v>652</v>
       </c>
       <c r="F394">
         <v>5</v>
@@ -24809,7 +24818,7 @@
         <v>296</v>
       </c>
       <c r="E395" t="s">
-        <v>654</v>
+        <v>653</v>
       </c>
       <c r="F395">
         <v>5</v>
@@ -24865,7 +24874,7 @@
         <v>298</v>
       </c>
       <c r="E396" t="s">
-        <v>655</v>
+        <v>654</v>
       </c>
       <c r="F396">
         <v>4</v>
@@ -24918,7 +24927,7 @@
         <v>84</v>
       </c>
       <c r="E397" t="s">
-        <v>656</v>
+        <v>655</v>
       </c>
       <c r="F397">
         <v>3</v>
@@ -24971,7 +24980,7 @@
         <v>301</v>
       </c>
       <c r="E398" t="s">
-        <v>657</v>
+        <v>656</v>
       </c>
       <c r="F398">
         <v>3</v>
@@ -25027,7 +25036,7 @@
         <v>209</v>
       </c>
       <c r="E399" t="s">
-        <v>658</v>
+        <v>657</v>
       </c>
       <c r="F399">
         <v>3</v>
@@ -25080,7 +25089,7 @@
         <v>194</v>
       </c>
       <c r="E400" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="F400">
         <v>4</v>
@@ -25133,7 +25142,7 @@
         <v>254</v>
       </c>
       <c r="E401" t="s">
-        <v>660</v>
+        <v>659</v>
       </c>
       <c r="F401">
         <v>5</v>
@@ -25186,7 +25195,7 @@
         <v>256</v>
       </c>
       <c r="E402" t="s">
-        <v>661</v>
+        <v>660</v>
       </c>
       <c r="F402">
         <v>3</v>
@@ -25239,7 +25248,7 @@
         <v>258</v>
       </c>
       <c r="E403" t="s">
-        <v>662</v>
+        <v>661</v>
       </c>
       <c r="F403">
         <v>4</v>
@@ -25295,7 +25304,7 @@
         <v>259</v>
       </c>
       <c r="E404" t="s">
-        <v>663</v>
+        <v>662</v>
       </c>
       <c r="F404">
         <v>4</v>
@@ -25351,7 +25360,7 @@
         <v>261</v>
       </c>
       <c r="E405" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="F405">
         <v>3</v>
@@ -25407,7 +25416,7 @@
         <v>263</v>
       </c>
       <c r="E406" t="s">
-        <v>665</v>
+        <v>664</v>
       </c>
       <c r="F406">
         <v>3</v>
@@ -25463,7 +25472,7 @@
         <v>265</v>
       </c>
       <c r="E407" t="s">
-        <v>666</v>
+        <v>665</v>
       </c>
       <c r="F407">
         <v>3</v>
@@ -25572,7 +25581,7 @@
         <v>269</v>
       </c>
       <c r="E409" t="s">
-        <v>667</v>
+        <v>666</v>
       </c>
       <c r="F409">
         <v>4</v>
@@ -25628,7 +25637,7 @@
         <v>271</v>
       </c>
       <c r="E410" t="s">
-        <v>668</v>
+        <v>667</v>
       </c>
       <c r="F410">
         <v>4</v>
@@ -25684,7 +25693,7 @@
         <v>177</v>
       </c>
       <c r="E411" t="s">
-        <v>669</v>
+        <v>668</v>
       </c>
       <c r="F411">
         <v>4</v>
@@ -25737,7 +25746,7 @@
         <v>274</v>
       </c>
       <c r="E412" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
       <c r="F412">
         <v>3</v>
@@ -25790,7 +25799,7 @@
         <v>276</v>
       </c>
       <c r="E413" t="s">
-        <v>671</v>
+        <v>670</v>
       </c>
       <c r="F413">
         <v>3</v>
@@ -25846,7 +25855,7 @@
         <v>213</v>
       </c>
       <c r="E414" t="s">
-        <v>672</v>
+        <v>671</v>
       </c>
       <c r="F414">
         <v>2</v>
@@ -25902,7 +25911,7 @@
         <v>211</v>
       </c>
       <c r="E415" t="s">
-        <v>673</v>
+        <v>672</v>
       </c>
       <c r="F415">
         <v>4</v>
@@ -25958,7 +25967,7 @@
         <v>280</v>
       </c>
       <c r="E416" t="s">
-        <v>674</v>
+        <v>673</v>
       </c>
       <c r="F416">
         <v>4</v>
@@ -26011,7 +26020,7 @@
         <v>282</v>
       </c>
       <c r="E417" t="s">
-        <v>675</v>
+        <v>674</v>
       </c>
       <c r="F417">
         <v>5</v>
@@ -26067,7 +26076,7 @@
         <v>284</v>
       </c>
       <c r="E418" t="s">
-        <v>676</v>
+        <v>675</v>
       </c>
       <c r="F418">
         <v>3</v>
@@ -26120,7 +26129,7 @@
         <v>286</v>
       </c>
       <c r="E419" t="s">
-        <v>677</v>
+        <v>676</v>
       </c>
       <c r="F419">
         <v>2</v>
@@ -26176,7 +26185,7 @@
         <v>288</v>
       </c>
       <c r="E420" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
       <c r="F420">
         <v>4</v>
@@ -26229,7 +26238,7 @@
         <v>290</v>
       </c>
       <c r="E421" t="s">
-        <v>679</v>
+        <v>678</v>
       </c>
       <c r="F421">
         <v>4</v>
@@ -26282,7 +26291,7 @@
         <v>292</v>
       </c>
       <c r="E422" t="s">
-        <v>680</v>
+        <v>679</v>
       </c>
       <c r="F422">
         <v>4</v>
@@ -26335,7 +26344,7 @@
         <v>294</v>
       </c>
       <c r="E423" t="s">
-        <v>681</v>
+        <v>680</v>
       </c>
       <c r="F423">
         <v>4</v>
@@ -26391,7 +26400,7 @@
         <v>296</v>
       </c>
       <c r="E424" t="s">
-        <v>682</v>
+        <v>681</v>
       </c>
       <c r="F424">
         <v>3</v>
@@ -26447,7 +26456,7 @@
         <v>298</v>
       </c>
       <c r="E425" t="s">
-        <v>683</v>
+        <v>682</v>
       </c>
       <c r="F425">
         <v>4</v>
@@ -26503,7 +26512,7 @@
         <v>84</v>
       </c>
       <c r="E426" t="s">
-        <v>684</v>
+        <v>683</v>
       </c>
       <c r="F426">
         <v>3</v>
@@ -26556,7 +26565,7 @@
         <v>301</v>
       </c>
       <c r="E427" t="s">
-        <v>685</v>
+        <v>684</v>
       </c>
       <c r="F427">
         <v>3</v>
@@ -26609,10 +26618,10 @@
         <v>6</v>
       </c>
       <c r="D428" t="s">
+        <v>685</v>
+      </c>
+      <c r="E428" t="s">
         <v>686</v>
-      </c>
-      <c r="E428" t="s">
-        <v>687</v>
       </c>
       <c r="F428">
         <v>2</v>
@@ -26665,7 +26674,7 @@
         <v>306</v>
       </c>
       <c r="E429" t="s">
-        <v>688</v>
+        <v>687</v>
       </c>
       <c r="F429">
         <v>4</v>
@@ -26718,7 +26727,7 @@
         <v>308</v>
       </c>
       <c r="E430" t="s">
-        <v>689</v>
+        <v>688</v>
       </c>
       <c r="F430">
         <v>4</v>
@@ -26939,7 +26948,7 @@
         <v>317</v>
       </c>
       <c r="E434" t="s">
-        <v>690</v>
+        <v>689</v>
       </c>
       <c r="F434">
         <v>5</v>
@@ -26995,7 +27004,7 @@
         <v>318</v>
       </c>
       <c r="E435" t="s">
-        <v>691</v>
+        <v>690</v>
       </c>
       <c r="F435">
         <v>4</v>
@@ -27051,7 +27060,7 @@
         <v>319</v>
       </c>
       <c r="E436" t="s">
-        <v>691</v>
+        <v>690</v>
       </c>
       <c r="F436">
         <v>4</v>
@@ -27107,7 +27116,7 @@
         <v>321</v>
       </c>
       <c r="E437" t="s">
-        <v>692</v>
+        <v>691</v>
       </c>
       <c r="F437">
         <v>4</v>
@@ -27163,7 +27172,7 @@
         <v>323</v>
       </c>
       <c r="E438" t="s">
-        <v>693</v>
+        <v>692</v>
       </c>
       <c r="F438">
         <v>4</v>
@@ -27219,7 +27228,7 @@
         <v>325</v>
       </c>
       <c r="E439" t="s">
-        <v>694</v>
+        <v>693</v>
       </c>
       <c r="F439">
         <v>4</v>
@@ -27275,7 +27284,7 @@
         <v>327</v>
       </c>
       <c r="E440" t="s">
-        <v>695</v>
+        <v>694</v>
       </c>
       <c r="F440">
         <v>3</v>
@@ -27331,7 +27340,7 @@
         <v>347</v>
       </c>
       <c r="E441" t="s">
-        <v>696</v>
+        <v>695</v>
       </c>
       <c r="F441">
         <v>4</v>
@@ -27384,7 +27393,7 @@
         <v>349</v>
       </c>
       <c r="E442" t="s">
-        <v>697</v>
+        <v>696</v>
       </c>
       <c r="F442">
         <v>5</v>
@@ -27434,10 +27443,10 @@
         <v>6</v>
       </c>
       <c r="D443" t="s">
-        <v>686</v>
+        <v>685</v>
       </c>
       <c r="E443" t="s">
-        <v>698</v>
+        <v>697</v>
       </c>
       <c r="F443">
         <v>2</v>
@@ -27490,7 +27499,7 @@
         <v>306</v>
       </c>
       <c r="E444" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
       <c r="F444">
         <v>5</v>
@@ -27543,7 +27552,7 @@
         <v>308</v>
       </c>
       <c r="E445" t="s">
-        <v>700</v>
+        <v>699</v>
       </c>
       <c r="F445">
         <v>4</v>
@@ -27596,7 +27605,7 @@
         <v>310</v>
       </c>
       <c r="E446" t="s">
-        <v>701</v>
+        <v>700</v>
       </c>
       <c r="F446">
         <v>4</v>
@@ -27652,7 +27661,7 @@
         <v>312</v>
       </c>
       <c r="E447" t="s">
-        <v>702</v>
+        <v>701</v>
       </c>
       <c r="F447">
         <v>5</v>
@@ -27708,7 +27717,7 @@
         <v>314</v>
       </c>
       <c r="E448" t="s">
-        <v>702</v>
+        <v>701</v>
       </c>
       <c r="F448">
         <v>4</v>
@@ -27764,7 +27773,7 @@
         <v>315</v>
       </c>
       <c r="E449" t="s">
-        <v>703</v>
+        <v>702</v>
       </c>
       <c r="F449">
         <v>3</v>
@@ -27820,7 +27829,7 @@
         <v>317</v>
       </c>
       <c r="E450" t="s">
-        <v>703</v>
+        <v>702</v>
       </c>
       <c r="F450">
         <v>4</v>
@@ -27876,7 +27885,7 @@
         <v>318</v>
       </c>
       <c r="E451" t="s">
-        <v>703</v>
+        <v>702</v>
       </c>
       <c r="F451">
         <v>4</v>
@@ -27932,7 +27941,7 @@
         <v>319</v>
       </c>
       <c r="E452" t="s">
-        <v>704</v>
+        <v>703</v>
       </c>
       <c r="F452">
         <v>4</v>
@@ -27988,7 +27997,7 @@
         <v>321</v>
       </c>
       <c r="E453" t="s">
-        <v>705</v>
+        <v>704</v>
       </c>
       <c r="F453">
         <v>3</v>
@@ -28044,7 +28053,7 @@
         <v>323</v>
       </c>
       <c r="E454" t="s">
-        <v>706</v>
+        <v>705</v>
       </c>
       <c r="F454">
         <v>3</v>
@@ -28100,7 +28109,7 @@
         <v>325</v>
       </c>
       <c r="E455" t="s">
-        <v>707</v>
+        <v>706</v>
       </c>
       <c r="F455">
         <v>5</v>
@@ -28156,7 +28165,7 @@
         <v>327</v>
       </c>
       <c r="E456" t="s">
-        <v>708</v>
+        <v>707</v>
       </c>
       <c r="F456">
         <v>3</v>
@@ -28212,7 +28221,7 @@
         <v>329</v>
       </c>
       <c r="E457" t="s">
-        <v>708</v>
+        <v>707</v>
       </c>
       <c r="F457">
         <v>4</v>
@@ -28268,7 +28277,7 @@
         <v>330</v>
       </c>
       <c r="E458" t="s">
-        <v>709</v>
+        <v>708</v>
       </c>
       <c r="F458">
         <v>4</v>
@@ -28324,7 +28333,7 @@
         <v>332</v>
       </c>
       <c r="E459" t="s">
-        <v>710</v>
+        <v>709</v>
       </c>
       <c r="F459">
         <v>5</v>
@@ -28380,7 +28389,7 @@
         <v>334</v>
       </c>
       <c r="E460" t="s">
-        <v>710</v>
+        <v>709</v>
       </c>
       <c r="F460">
         <v>4</v>
@@ -28436,7 +28445,7 @@
         <v>335</v>
       </c>
       <c r="E461" t="s">
-        <v>711</v>
+        <v>710</v>
       </c>
       <c r="F461">
         <v>3</v>
@@ -28492,7 +28501,7 @@
         <v>337</v>
       </c>
       <c r="E462" t="s">
-        <v>712</v>
+        <v>711</v>
       </c>
       <c r="F462">
         <v>4</v>
@@ -28548,7 +28557,7 @@
         <v>339</v>
       </c>
       <c r="E463" t="s">
-        <v>713</v>
+        <v>712</v>
       </c>
       <c r="F463">
         <v>3</v>
@@ -28604,7 +28613,7 @@
         <v>340</v>
       </c>
       <c r="E464" t="s">
-        <v>714</v>
+        <v>713</v>
       </c>
       <c r="F464">
         <v>3</v>
@@ -28657,7 +28666,7 @@
         <v>342</v>
       </c>
       <c r="E465" t="s">
-        <v>715</v>
+        <v>714</v>
       </c>
       <c r="F465">
         <v>4</v>
@@ -28710,7 +28719,7 @@
         <v>345</v>
       </c>
       <c r="E466" t="s">
-        <v>716</v>
+        <v>715</v>
       </c>
       <c r="F466">
         <v>3</v>
@@ -28763,7 +28772,7 @@
         <v>347</v>
       </c>
       <c r="E467" t="s">
-        <v>717</v>
+        <v>716</v>
       </c>
       <c r="F467">
         <v>5</v>
@@ -28816,7 +28825,7 @@
         <v>349</v>
       </c>
       <c r="E468" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
       <c r="F468">
         <v>5</v>
@@ -28869,7 +28878,7 @@
         <v>351</v>
       </c>
       <c r="E469" t="s">
-        <v>719</v>
+        <v>718</v>
       </c>
       <c r="F469">
         <v>5</v>
@@ -28922,7 +28931,7 @@
         <v>353</v>
       </c>
       <c r="E470" t="s">
-        <v>720</v>
+        <v>719</v>
       </c>
       <c r="F470">
         <v>4</v>
@@ -28975,7 +28984,7 @@
         <v>356</v>
       </c>
       <c r="E471" t="s">
-        <v>720</v>
+        <v>719</v>
       </c>
       <c r="F471">
         <v>4</v>
@@ -29140,7 +29149,7 @@
         <v>362</v>
       </c>
       <c r="E474" t="s">
-        <v>721</v>
+        <v>720</v>
       </c>
       <c r="F474">
         <v>3</v>
@@ -29196,7 +29205,7 @@
         <v>364</v>
       </c>
       <c r="E475" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="F475">
         <v>3</v>
@@ -29249,7 +29258,7 @@
         <v>366</v>
       </c>
       <c r="E476" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
       <c r="F476">
         <v>3</v>
@@ -29302,7 +29311,7 @@
         <v>368</v>
       </c>
       <c r="E477" t="s">
-        <v>724</v>
+        <v>723</v>
       </c>
       <c r="F477">
         <v>3</v>
@@ -29355,7 +29364,7 @@
         <v>370</v>
       </c>
       <c r="E478" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="F478">
         <v>4</v>
@@ -29408,7 +29417,7 @@
         <v>372</v>
       </c>
       <c r="E479" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
       <c r="F479">
         <v>3</v>
@@ -29458,7 +29467,7 @@
         <v>347</v>
       </c>
       <c r="E480" t="s">
-        <v>727</v>
+        <v>726</v>
       </c>
       <c r="F480">
         <v>3</v>
@@ -29485,7 +29494,7 @@
         <v>50.92</v>
       </c>
       <c r="O480" t="s">
-        <v>728</v>
+        <v>727</v>
       </c>
       <c r="P480">
         <v>0</v>
@@ -29511,7 +29520,7 @@
         <v>345</v>
       </c>
       <c r="E481" t="s">
-        <v>729</v>
+        <v>728</v>
       </c>
       <c r="F481">
         <v>4</v>
@@ -29564,7 +29573,7 @@
         <v>377</v>
       </c>
       <c r="E482" t="s">
-        <v>730</v>
+        <v>729</v>
       </c>
       <c r="F482">
         <v>5</v>
@@ -29620,7 +29629,7 @@
         <v>379</v>
       </c>
       <c r="E483" t="s">
-        <v>731</v>
+        <v>730</v>
       </c>
       <c r="F483">
         <v>4</v>
@@ -29676,7 +29685,7 @@
         <v>381</v>
       </c>
       <c r="E484" t="s">
-        <v>732</v>
+        <v>731</v>
       </c>
       <c r="F484">
         <v>5</v>
@@ -29732,7 +29741,7 @@
         <v>383</v>
       </c>
       <c r="E485" t="s">
-        <v>733</v>
+        <v>732</v>
       </c>
       <c r="F485">
         <v>5</v>
@@ -29788,7 +29797,7 @@
         <v>384</v>
       </c>
       <c r="E486" t="s">
-        <v>734</v>
+        <v>733</v>
       </c>
       <c r="F486">
         <v>5</v>
@@ -29844,7 +29853,7 @@
         <v>385</v>
       </c>
       <c r="E487" t="s">
-        <v>735</v>
+        <v>734</v>
       </c>
       <c r="F487">
         <v>3</v>
@@ -29900,7 +29909,7 @@
         <v>387</v>
       </c>
       <c r="E488" t="s">
-        <v>736</v>
+        <v>735</v>
       </c>
       <c r="F488">
         <v>4</v>
@@ -29953,7 +29962,7 @@
         <v>389</v>
       </c>
       <c r="E489" t="s">
-        <v>737</v>
+        <v>736</v>
       </c>
       <c r="F489">
         <v>4</v>
@@ -30006,7 +30015,7 @@
         <v>213</v>
       </c>
       <c r="E490" t="s">
-        <v>738</v>
+        <v>737</v>
       </c>
       <c r="F490">
         <v>4</v>
@@ -30059,7 +30068,7 @@
         <v>211</v>
       </c>
       <c r="E491" t="s">
-        <v>739</v>
+        <v>738</v>
       </c>
       <c r="F491">
         <v>4</v>
@@ -30109,10 +30118,10 @@
         <v>7</v>
       </c>
       <c r="D492" t="s">
+        <v>739</v>
+      </c>
+      <c r="E492" t="s">
         <v>740</v>
-      </c>
-      <c r="E492" t="s">
-        <v>741</v>
       </c>
       <c r="F492">
         <v>4</v>
@@ -30165,7 +30174,7 @@
         <v>395</v>
       </c>
       <c r="E493" t="s">
-        <v>742</v>
+        <v>741</v>
       </c>
       <c r="F493">
         <v>4</v>
@@ -30218,7 +30227,7 @@
         <v>397</v>
       </c>
       <c r="E494" t="s">
-        <v>743</v>
+        <v>742</v>
       </c>
       <c r="F494">
         <v>3</v>
@@ -30271,7 +30280,7 @@
         <v>399</v>
       </c>
       <c r="E495" t="s">
-        <v>744</v>
+        <v>743</v>
       </c>
       <c r="F495">
         <v>4</v>
@@ -30324,7 +30333,7 @@
         <v>401</v>
       </c>
       <c r="E496" t="s">
-        <v>745</v>
+        <v>744</v>
       </c>
       <c r="F496">
         <v>4</v>
@@ -30377,7 +30386,7 @@
         <v>403</v>
       </c>
       <c r="E497" t="s">
-        <v>746</v>
+        <v>745</v>
       </c>
       <c r="F497">
         <v>4</v>
@@ -30430,7 +30439,7 @@
         <v>405</v>
       </c>
       <c r="E498" t="s">
-        <v>747</v>
+        <v>746</v>
       </c>
       <c r="F498">
         <v>5</v>
@@ -30486,7 +30495,7 @@
         <v>351</v>
       </c>
       <c r="E499" t="s">
-        <v>748</v>
+        <v>747</v>
       </c>
       <c r="F499">
         <v>4</v>
@@ -30542,7 +30551,7 @@
         <v>353</v>
       </c>
       <c r="E500" t="s">
-        <v>749</v>
+        <v>748</v>
       </c>
       <c r="F500">
         <v>3</v>
@@ -30598,7 +30607,7 @@
         <v>356</v>
       </c>
       <c r="E501" t="s">
-        <v>749</v>
+        <v>748</v>
       </c>
       <c r="F501">
         <v>4</v>
@@ -30654,7 +30663,7 @@
         <v>357</v>
       </c>
       <c r="E502" t="s">
-        <v>750</v>
+        <v>749</v>
       </c>
       <c r="F502">
         <v>3</v>
@@ -30707,7 +30716,7 @@
         <v>359</v>
       </c>
       <c r="E503" t="s">
-        <v>751</v>
+        <v>750</v>
       </c>
       <c r="F503">
         <v>3</v>
@@ -30763,7 +30772,7 @@
         <v>362</v>
       </c>
       <c r="E504" t="s">
-        <v>751</v>
+        <v>750</v>
       </c>
       <c r="F504">
         <v>3</v>
@@ -30819,7 +30828,7 @@
         <v>364</v>
       </c>
       <c r="E505" t="s">
-        <v>752</v>
+        <v>751</v>
       </c>
       <c r="F505">
         <v>1</v>
@@ -30869,7 +30878,7 @@
         <v>366</v>
       </c>
       <c r="E506" t="s">
-        <v>753</v>
+        <v>752</v>
       </c>
       <c r="F506">
         <v>3</v>
@@ -30922,7 +30931,7 @@
         <v>368</v>
       </c>
       <c r="E507" t="s">
-        <v>754</v>
+        <v>753</v>
       </c>
       <c r="F507">
         <v>3</v>
@@ -30975,7 +30984,7 @@
         <v>370</v>
       </c>
       <c r="E508" t="s">
-        <v>755</v>
+        <v>754</v>
       </c>
       <c r="F508">
         <v>3</v>
@@ -31028,7 +31037,7 @@
         <v>372</v>
       </c>
       <c r="E509" t="s">
-        <v>756</v>
+        <v>755</v>
       </c>
       <c r="F509">
         <v>3</v>
@@ -31081,7 +31090,7 @@
         <v>347</v>
       </c>
       <c r="E510" t="s">
-        <v>757</v>
+        <v>756</v>
       </c>
       <c r="F510">
         <v>4</v>
@@ -31134,7 +31143,7 @@
         <v>345</v>
       </c>
       <c r="E511" t="s">
-        <v>758</v>
+        <v>757</v>
       </c>
       <c r="F511">
         <v>3</v>
@@ -31187,7 +31196,7 @@
         <v>377</v>
       </c>
       <c r="E512" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="F512">
         <v>5</v>
@@ -31243,7 +31252,7 @@
         <v>379</v>
       </c>
       <c r="E513" t="s">
-        <v>760</v>
+        <v>759</v>
       </c>
       <c r="F513">
         <v>3</v>
@@ -31299,7 +31308,7 @@
         <v>381</v>
       </c>
       <c r="E514" t="s">
-        <v>761</v>
+        <v>760</v>
       </c>
       <c r="F514">
         <v>4</v>
@@ -31355,7 +31364,7 @@
         <v>383</v>
       </c>
       <c r="E515" t="s">
-        <v>762</v>
+        <v>761</v>
       </c>
       <c r="F515">
         <v>3</v>
@@ -31411,7 +31420,7 @@
         <v>384</v>
       </c>
       <c r="E516" t="s">
-        <v>763</v>
+        <v>762</v>
       </c>
       <c r="F516">
         <v>3</v>
@@ -31467,7 +31476,7 @@
         <v>385</v>
       </c>
       <c r="E517" t="s">
-        <v>764</v>
+        <v>763</v>
       </c>
       <c r="F517">
         <v>4</v>
@@ -31523,7 +31532,7 @@
         <v>387</v>
       </c>
       <c r="E518" t="s">
-        <v>765</v>
+        <v>764</v>
       </c>
       <c r="F518">
         <v>5</v>
@@ -31576,7 +31585,7 @@
         <v>389</v>
       </c>
       <c r="E519" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="F519">
         <v>5</v>
@@ -31629,7 +31638,7 @@
         <v>213</v>
       </c>
       <c r="E520" t="s">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="F520">
         <v>4</v>
@@ -31682,7 +31691,7 @@
         <v>211</v>
       </c>
       <c r="E521" t="s">
-        <v>768</v>
+        <v>767</v>
       </c>
       <c r="F521">
         <v>4</v>
@@ -31732,10 +31741,10 @@
         <v>7</v>
       </c>
       <c r="D522" t="s">
-        <v>740</v>
+        <v>739</v>
       </c>
       <c r="E522" t="s">
-        <v>769</v>
+        <v>768</v>
       </c>
       <c r="F522">
         <v>5</v>
@@ -31788,7 +31797,7 @@
         <v>395</v>
       </c>
       <c r="E523" t="s">
-        <v>770</v>
+        <v>769</v>
       </c>
       <c r="F523">
         <v>3</v>
@@ -31841,7 +31850,7 @@
         <v>397</v>
       </c>
       <c r="E524" t="s">
-        <v>771</v>
+        <v>770</v>
       </c>
       <c r="F524">
         <v>3</v>
@@ -31894,7 +31903,7 @@
         <v>399</v>
       </c>
       <c r="E525" t="s">
-        <v>772</v>
+        <v>771</v>
       </c>
       <c r="F525">
         <v>4</v>
@@ -31944,7 +31953,7 @@
         <v>401</v>
       </c>
       <c r="E526" t="s">
-        <v>773</v>
+        <v>772</v>
       </c>
       <c r="F526">
         <v>5</v>
@@ -31997,7 +32006,7 @@
         <v>403</v>
       </c>
       <c r="E527" t="s">
-        <v>774</v>
+        <v>773</v>
       </c>
       <c r="F527">
         <v>4</v>
@@ -32050,7 +32059,7 @@
         <v>405</v>
       </c>
       <c r="E528" t="s">
-        <v>775</v>
+        <v>774</v>
       </c>
       <c r="F528">
         <v>5</v>
@@ -32178,7 +32187,7 @@
         <v>5</v>
       </c>
       <c r="J530">
-        <f t="shared" ref="J530:J551" si="4">SUM(F530:I530)</f>
+        <f t="shared" ref="J530:J550" si="4">SUM(F530:I530)</f>
         <v>16</v>
       </c>
       <c r="K530">
@@ -33570,11 +33579,11 @@
         <v/>
       </c>
       <c r="P2" t="str">
-        <f>IFERROR(AVERAGE('Results_qwen2.5_latest'!T2:T10000),"")</f>
+        <f>IFERROR(AVERAGE('Results_qwen2.5_latest'!#REF!),"")</f>
         <v/>
       </c>
       <c r="Q2">
-        <f>IFERROR(COUNTIF('Results_qwen2.5_latest'!U2:U10000,"&lt;&gt;")/COUNTA('Results_qwen2.5_latest'!A2:A10000)*100,"")</f>
+        <f>IFERROR(COUNTIF('Results_qwen2.5_latest'!T2:T10000,"&lt;&gt;")/COUNTA('Results_qwen2.5_latest'!A2:A10000)*100,"")</f>
         <v>0</v>
       </c>
     </row>

</xml_diff>